<commit_message>
Implemented zebralogic to SMT program and finished all zebralogic of Python.
</commit_message>
<xml_diff>
--- a/output/Plan/gpt-5-2025-08-07/task_analysis_results_singlepass_Plan_gpt-5-2025-08-07_calendar.xlsx
+++ b/output/Plan/gpt-5-2025-08-07/task_analysis_results_singlepass_Plan_gpt-5-2025-08-07_calendar.xlsx
@@ -1796,18 +1796,18 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exact match</t>
+          <t>Correct plan (constraints satisfied)</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>{"time_range": "{12:00:13:00}", "day": "Tuesday"}</t>
+          <t>{"time_range": "{12:30:13:30}", "day": "Tuesday"}</t>
         </is>
       </c>
     </row>
@@ -2608,18 +2608,18 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Failed to solve within max passes</t>
+          <t>Exact match</t>
         </is>
       </c>
       <c r="E40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Understood. Please provide the specific participants, their schedules, the meeting duration, work hour constraints, and any time preferences so I can propose a time.</t>
+          <t>{"time_range": "{13:00:14:00}", "day": "Monday"}</t>
         </is>
       </c>
     </row>
@@ -3159,18 +3159,18 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Exact match</t>
+          <t>Correct plan (constraints satisfied)</t>
         </is>
       </c>
       <c r="E59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F59" t="b">
         <v>1</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>{"time_range": "{12:30:13:00}", "day": "Monday"}</t>
+          <t>{"time_range": "{11:00:11:30}", "day": "Wednesday"}</t>
         </is>
       </c>
     </row>
@@ -3362,18 +3362,18 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Exact match</t>
+          <t>Correct plan (constraints satisfied)</t>
         </is>
       </c>
       <c r="E66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F66" t="b">
         <v>1</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>{"time_range": "{12:00:13:00}", "day": "Wednesday"}</t>
+          <t>{"time_range":"{12:30:13:30}","day":"Wednesday"}</t>
         </is>
       </c>
     </row>

</xml_diff>